<commit_message>
jhyal dhoka break down in same file for hawa huri
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/hawa huri jhyal/water tank 2082_2083.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/hawa huri jhyal/water tank 2082_2083.xlsx
@@ -1,36 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\बजेट माग estimate\nagar bhaipari and estimate misc\hawa huri jhyal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33AC54EF-B0AB-49D7-9717-AB327D104429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B60F61-A392-48EA-9A20-B23EDF0ABE30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ESTIMATE" sheetId="25" state="hidden" r:id="rId1"/>
     <sheet name="WCR" sheetId="27" state="hidden" r:id="rId2"/>
     <sheet name="me" sheetId="29" state="hidden" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="30" state="hidden" r:id="rId4"/>
-    <sheet name="&lt;1000000" sheetId="31" r:id="rId5"/>
-    <sheet name="&lt;1000000 (2)" sheetId="32" r:id="rId6"/>
+    <sheet name="&lt;1000000" sheetId="31" state="hidden" r:id="rId5"/>
+    <sheet name="&lt;1000000 (2)" sheetId="32" state="hidden" r:id="rId6"/>
+    <sheet name="&lt;1000000 (3)" sheetId="33" r:id="rId7"/>
+    <sheet name="&lt;1000000 (4)" sheetId="34" r:id="rId8"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId7"/>
-    <externalReference r:id="rId8"/>
+    <externalReference r:id="rId9"/>
+    <externalReference r:id="rId10"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'&lt;1000000'!$A$1:$L$24</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'&lt;1000000 (2)'!$A$1:$L$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'&lt;1000000 (3)'!$A$1:$L$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'&lt;1000000 (4)'!$A$1:$L$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">ESTIMATE!$A$1:$L$71</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">me!$A$1:$L$162</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'&lt;1000000'!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'&lt;1000000 (2)'!$1:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'&lt;1000000 (3)'!$1:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'&lt;1000000 (4)'!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">ESTIMATE!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">me!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">WCR!$1:$11</definedName>
@@ -111,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="183">
   <si>
     <t>S.N.</t>
   </si>
@@ -802,6 +808,47 @@
   </si>
   <si>
     <t>-at kitchen</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Project:-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Preeti"/>
+      </rPr>
+      <t>lalaw ‰ofn9f]sf dd{t sfo{ j8f sfof{no</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Project:-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Preeti"/>
+      </rPr>
+      <t>lalaw ‰ofn9f]sf dd{t sfo{ :jf:Yo rf}sL</t>
+    </r>
+  </si>
+  <si>
+    <t>Date: 2083/02/02</t>
   </si>
 </sst>
 </file>
@@ -3238,6 +3285,10 @@
     <xf numFmtId="0" fontId="49" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="89" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="182" fontId="51" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="43" fontId="51" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3260,6 +3311,24 @@
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="63" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3275,24 +3344,6 @@
     <xf numFmtId="0" fontId="65" fillId="32" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="63" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="43" fontId="51" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3322,10 +3373,6 @@
     </xf>
     <xf numFmtId="0" fontId="82" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="89" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="182" fontId="51" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="759">
@@ -4704,68 +4751,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="162" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="160"/>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160"/>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160"/>
-      <c r="I1" s="160"/>
-      <c r="J1" s="160"/>
-      <c r="K1" s="160"/>
-      <c r="L1" s="160"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
     </row>
     <row r="2" spans="1:18" ht="20.25">
-      <c r="A2" s="161" t="s">
+      <c r="A2" s="163" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="161"/>
-      <c r="C2" s="161"/>
-      <c r="D2" s="161"/>
-      <c r="E2" s="161"/>
-      <c r="F2" s="161"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="161"/>
-      <c r="I2" s="161"/>
-      <c r="J2" s="161"/>
-      <c r="K2" s="161"/>
-      <c r="L2" s="161"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
+      <c r="H2" s="163"/>
+      <c r="I2" s="163"/>
+      <c r="J2" s="163"/>
+      <c r="K2" s="163"/>
+      <c r="L2" s="163"/>
     </row>
     <row r="3" spans="1:18">
-      <c r="A3" s="160" t="s">
+      <c r="A3" s="162" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="160"/>
-      <c r="C3" s="160"/>
-      <c r="D3" s="160"/>
-      <c r="E3" s="160"/>
-      <c r="F3" s="160"/>
-      <c r="G3" s="160"/>
-      <c r="H3" s="160"/>
-      <c r="I3" s="160"/>
-      <c r="J3" s="160"/>
-      <c r="K3" s="160"/>
-      <c r="L3" s="160"/>
+      <c r="B3" s="162"/>
+      <c r="C3" s="162"/>
+      <c r="D3" s="162"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="162"/>
+      <c r="G3" s="162"/>
+      <c r="H3" s="162"/>
+      <c r="I3" s="162"/>
+      <c r="J3" s="162"/>
+      <c r="K3" s="162"/>
+      <c r="L3" s="162"/>
     </row>
     <row r="4" spans="1:18">
-      <c r="A4" s="162" t="s">
+      <c r="A4" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="162"/>
-      <c r="C4" s="162"/>
-      <c r="D4" s="162"/>
-      <c r="E4" s="162"/>
-      <c r="F4" s="162"/>
-      <c r="G4" s="162"/>
-      <c r="H4" s="162"/>
-      <c r="I4" s="162"/>
-      <c r="J4" s="162"/>
-      <c r="K4" s="162"/>
-      <c r="L4" s="162"/>
+      <c r="B4" s="164"/>
+      <c r="C4" s="164"/>
+      <c r="D4" s="164"/>
+      <c r="E4" s="164"/>
+      <c r="F4" s="164"/>
+      <c r="G4" s="164"/>
+      <c r="H4" s="164"/>
+      <c r="I4" s="164"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="164"/>
+      <c r="L4" s="164"/>
     </row>
     <row r="5" spans="1:18" ht="19.5">
       <c r="A5" s="6"/>
@@ -4776,33 +4823,33 @@
         <v>93</v>
       </c>
       <c r="H5" s="6"/>
-      <c r="K5" s="163" t="s">
+      <c r="K5" s="165" t="s">
         <v>69</v>
       </c>
-      <c r="L5" s="163"/>
+      <c r="L5" s="165"/>
     </row>
     <row r="6" spans="1:18">
-      <c r="B6" s="164" t="s">
+      <c r="B6" s="166" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="164"/>
-      <c r="D6" s="164"/>
-      <c r="E6" s="164"/>
-      <c r="F6" s="164"/>
-      <c r="G6" s="164"/>
+      <c r="C6" s="166"/>
+      <c r="D6" s="166"/>
+      <c r="E6" s="166"/>
+      <c r="F6" s="166"/>
+      <c r="G6" s="166"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="165" t="s">
+      <c r="I6" s="167" t="s">
         <v>100</v>
       </c>
-      <c r="J6" s="165"/>
-      <c r="K6" s="165"/>
-      <c r="L6" s="165"/>
-      <c r="O6" s="165" t="s">
+      <c r="J6" s="167"/>
+      <c r="K6" s="167"/>
+      <c r="L6" s="167"/>
+      <c r="O6" s="167" t="s">
         <v>70</v>
       </c>
-      <c r="P6" s="165"/>
-      <c r="Q6" s="165"/>
-      <c r="R6" s="165"/>
+      <c r="P6" s="167"/>
+      <c r="Q6" s="167"/>
+      <c r="R6" s="167"/>
     </row>
     <row r="7" spans="1:18" ht="17.25" thickBot="1">
       <c r="C7" s="5"/>
@@ -6372,60 +6419,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="171" t="s">
+      <c r="A1" s="168" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="171"/>
-      <c r="C1" s="171"/>
-      <c r="D1" s="171"/>
-      <c r="E1" s="171"/>
-      <c r="F1" s="171"/>
-      <c r="G1" s="171"/>
-      <c r="H1" s="171"/>
-      <c r="I1" s="171"/>
-      <c r="J1" s="171"/>
+      <c r="B1" s="168"/>
+      <c r="C1" s="168"/>
+      <c r="D1" s="168"/>
+      <c r="E1" s="168"/>
+      <c r="F1" s="168"/>
+      <c r="G1" s="168"/>
+      <c r="H1" s="168"/>
+      <c r="I1" s="168"/>
+      <c r="J1" s="168"/>
     </row>
     <row r="2" spans="1:10" ht="25.5">
-      <c r="A2" s="172" t="s">
+      <c r="A2" s="169" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="172"/>
-      <c r="C2" s="172"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="F2" s="172"/>
-      <c r="G2" s="172"/>
-      <c r="H2" s="172"/>
-      <c r="I2" s="172"/>
-      <c r="J2" s="172"/>
+      <c r="B2" s="169"/>
+      <c r="C2" s="169"/>
+      <c r="D2" s="169"/>
+      <c r="E2" s="169"/>
+      <c r="F2" s="169"/>
+      <c r="G2" s="169"/>
+      <c r="H2" s="169"/>
+      <c r="I2" s="169"/>
+      <c r="J2" s="169"/>
     </row>
     <row r="3" spans="1:10" ht="18.75">
-      <c r="A3" s="173" t="s">
+      <c r="A3" s="170" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="173"/>
-      <c r="C3" s="173"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="173"/>
-      <c r="F3" s="173"/>
-      <c r="G3" s="173"/>
-      <c r="H3" s="173"/>
-      <c r="I3" s="173"/>
-      <c r="J3" s="173"/>
+      <c r="B3" s="170"/>
+      <c r="C3" s="170"/>
+      <c r="D3" s="170"/>
+      <c r="E3" s="170"/>
+      <c r="F3" s="170"/>
+      <c r="G3" s="170"/>
+      <c r="H3" s="170"/>
+      <c r="I3" s="170"/>
+      <c r="J3" s="170"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="174" t="s">
+      <c r="A4" s="171" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="174"/>
-      <c r="C4" s="174"/>
-      <c r="D4" s="174"/>
-      <c r="E4" s="174"/>
-      <c r="F4" s="174"/>
-      <c r="G4" s="174"/>
-      <c r="H4" s="174"/>
-      <c r="I4" s="174"/>
-      <c r="J4" s="174"/>
+      <c r="B4" s="171"/>
+      <c r="C4" s="171"/>
+      <c r="D4" s="171"/>
+      <c r="E4" s="171"/>
+      <c r="F4" s="171"/>
+      <c r="G4" s="171"/>
+      <c r="H4" s="171"/>
+      <c r="I4" s="171"/>
+      <c r="J4" s="171"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="37"/>
@@ -6444,33 +6491,33 @@
         <v>55</v>
       </c>
       <c r="B6" s="31"/>
-      <c r="C6" s="175" t="e">
+      <c r="C6" s="172" t="e">
         <f>E51</f>
         <v>#REF!</v>
       </c>
-      <c r="D6" s="176"/>
+      <c r="D6" s="173"/>
       <c r="E6" s="31"/>
       <c r="F6" s="31"/>
       <c r="G6" s="31" t="s">
         <v>56</v>
       </c>
       <c r="H6" s="31"/>
-      <c r="I6" s="175" t="e">
+      <c r="I6" s="172" t="e">
         <f>H51</f>
         <v>#REF!</v>
       </c>
-      <c r="J6" s="176"/>
+      <c r="J6" s="173"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="32"/>
       <c r="B7" s="32"/>
-      <c r="C7" s="166"/>
-      <c r="D7" s="166"/>
-      <c r="E7" s="166"/>
-      <c r="F7" s="166"/>
-      <c r="H7" s="167"/>
-      <c r="I7" s="167"/>
-      <c r="J7" s="167"/>
+      <c r="C7" s="174"/>
+      <c r="D7" s="174"/>
+      <c r="E7" s="174"/>
+      <c r="F7" s="174"/>
+      <c r="H7" s="175"/>
+      <c r="I7" s="175"/>
+      <c r="J7" s="175"/>
     </row>
     <row r="8" spans="1:10" ht="16.5">
       <c r="A8" t="s">
@@ -6497,32 +6544,32 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="168" t="s">
+      <c r="A10" s="176" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="168" t="s">
+      <c r="B10" s="176" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="170" t="s">
+      <c r="C10" s="178" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="170"/>
-      <c r="E10" s="170"/>
-      <c r="F10" s="170" t="s">
+      <c r="D10" s="178"/>
+      <c r="E10" s="178"/>
+      <c r="F10" s="178" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="170"/>
-      <c r="H10" s="170"/>
-      <c r="I10" s="168" t="s">
+      <c r="G10" s="178"/>
+      <c r="H10" s="178"/>
+      <c r="I10" s="176" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="168" t="s">
+      <c r="J10" s="176" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="169"/>
-      <c r="B11" s="169"/>
+      <c r="A11" s="177"/>
+      <c r="B11" s="177"/>
       <c r="C11" s="39" t="s">
         <v>64</v>
       </c>
@@ -6541,8 +6588,8 @@
       <c r="H11" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="I11" s="169"/>
-      <c r="J11" s="169"/>
+      <c r="I11" s="177"/>
+      <c r="J11" s="177"/>
     </row>
     <row r="12" spans="1:10" ht="15.75">
       <c r="A12" s="47">
@@ -7469,12 +7516,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="H7:J7"/>
@@ -7484,6 +7525,12 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I10:I11"/>
     <mergeCell ref="J10:J11"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -7520,68 +7567,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="162" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="160"/>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160"/>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160"/>
-      <c r="I1" s="160"/>
-      <c r="J1" s="160"/>
-      <c r="K1" s="160"/>
-      <c r="L1" s="160"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
     </row>
     <row r="2" spans="1:12" ht="20.25">
-      <c r="A2" s="161" t="s">
+      <c r="A2" s="163" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="161"/>
-      <c r="C2" s="161"/>
-      <c r="D2" s="161"/>
-      <c r="E2" s="161"/>
-      <c r="F2" s="161"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="161"/>
-      <c r="I2" s="161"/>
-      <c r="J2" s="161"/>
-      <c r="K2" s="161"/>
-      <c r="L2" s="161"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
+      <c r="H2" s="163"/>
+      <c r="I2" s="163"/>
+      <c r="J2" s="163"/>
+      <c r="K2" s="163"/>
+      <c r="L2" s="163"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="160" t="s">
+      <c r="A3" s="162" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="160"/>
-      <c r="C3" s="160"/>
-      <c r="D3" s="160"/>
-      <c r="E3" s="160"/>
-      <c r="F3" s="160"/>
-      <c r="G3" s="160"/>
-      <c r="H3" s="160"/>
-      <c r="I3" s="160"/>
-      <c r="J3" s="160"/>
-      <c r="K3" s="160"/>
-      <c r="L3" s="160"/>
+      <c r="B3" s="162"/>
+      <c r="C3" s="162"/>
+      <c r="D3" s="162"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="162"/>
+      <c r="G3" s="162"/>
+      <c r="H3" s="162"/>
+      <c r="I3" s="162"/>
+      <c r="J3" s="162"/>
+      <c r="K3" s="162"/>
+      <c r="L3" s="162"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="162" t="s">
+      <c r="A4" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="162"/>
-      <c r="C4" s="162"/>
-      <c r="D4" s="162"/>
-      <c r="E4" s="162"/>
-      <c r="F4" s="162"/>
-      <c r="G4" s="162"/>
-      <c r="H4" s="162"/>
-      <c r="I4" s="162"/>
-      <c r="J4" s="162"/>
-      <c r="K4" s="162"/>
-      <c r="L4" s="162"/>
+      <c r="B4" s="164"/>
+      <c r="C4" s="164"/>
+      <c r="D4" s="164"/>
+      <c r="E4" s="164"/>
+      <c r="F4" s="164"/>
+      <c r="G4" s="164"/>
+      <c r="H4" s="164"/>
+      <c r="I4" s="164"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="164"/>
+      <c r="L4" s="164"/>
     </row>
     <row r="5" spans="1:12" ht="20.25">
       <c r="A5" s="6"/>
@@ -7589,27 +7636,27 @@
         <v>168</v>
       </c>
       <c r="H5" s="6"/>
-      <c r="K5" s="163" t="s">
+      <c r="K5" s="165" t="s">
         <v>101</v>
       </c>
-      <c r="L5" s="163"/>
+      <c r="L5" s="165"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="B6" s="164" t="s">
+      <c r="B6" s="166" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="164"/>
-      <c r="D6" s="164"/>
-      <c r="E6" s="164"/>
-      <c r="F6" s="164"/>
-      <c r="G6" s="164"/>
+      <c r="C6" s="166"/>
+      <c r="D6" s="166"/>
+      <c r="E6" s="166"/>
+      <c r="F6" s="166"/>
+      <c r="G6" s="166"/>
       <c r="H6" s="113"/>
-      <c r="I6" s="165" t="s">
+      <c r="I6" s="167" t="s">
         <v>167</v>
       </c>
-      <c r="J6" s="165"/>
-      <c r="K6" s="165"/>
-      <c r="L6" s="165"/>
+      <c r="J6" s="167"/>
+      <c r="K6" s="167"/>
+      <c r="L6" s="167"/>
     </row>
     <row r="7" spans="1:12">
       <c r="C7" s="5"/>
@@ -10767,10 +10814,10 @@
       <c r="C156" s="124" t="s">
         <v>12</v>
       </c>
-      <c r="D156" s="178" t="s">
+      <c r="D156" s="180" t="s">
         <v>71</v>
       </c>
-      <c r="E156" s="178"/>
+      <c r="E156" s="180"/>
       <c r="F156" s="124" t="s">
         <v>72</v>
       </c>
@@ -10780,11 +10827,11 @@
       <c r="C157" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D157" s="158">
+      <c r="D157" s="160">
         <f>+K154</f>
         <v>877810.68270516139</v>
       </c>
-      <c r="E157" s="158"/>
+      <c r="E157" s="160"/>
       <c r="F157" s="152"/>
       <c r="H157" s="64"/>
     </row>
@@ -10792,10 +10839,10 @@
       <c r="C158" s="134" t="s">
         <v>14</v>
       </c>
-      <c r="D158" s="158">
+      <c r="D158" s="160">
         <v>200000</v>
       </c>
-      <c r="E158" s="158"/>
+      <c r="E158" s="160"/>
       <c r="F158" s="153">
         <v>100</v>
       </c>
@@ -10805,11 +10852,11 @@
       <c r="C159" s="134" t="s">
         <v>19</v>
       </c>
-      <c r="D159" s="158">
+      <c r="D159" s="160">
         <f>0.95*D158</f>
         <v>190000</v>
       </c>
-      <c r="E159" s="158"/>
+      <c r="E159" s="160"/>
       <c r="F159" s="153">
         <f>D159/D157*100</f>
         <v>21.644758231293604</v>
@@ -10820,11 +10867,11 @@
       <c r="C160" s="134" t="s">
         <v>15</v>
       </c>
-      <c r="D160" s="158">
+      <c r="D160" s="160">
         <f>D157-D159</f>
         <v>687810.68270516139</v>
       </c>
-      <c r="E160" s="158"/>
+      <c r="E160" s="160"/>
       <c r="F160" s="153">
         <f>D160/D158*100</f>
         <v>343.90534135258071</v>
@@ -10835,11 +10882,11 @@
       <c r="C161" s="134" t="s">
         <v>20</v>
       </c>
-      <c r="D161" s="158">
+      <c r="D161" s="160">
         <f>F161*D158/100</f>
         <v>4000</v>
       </c>
-      <c r="E161" s="158"/>
+      <c r="E161" s="160"/>
       <c r="F161" s="153">
         <v>2</v>
       </c>
@@ -10849,11 +10896,11 @@
       <c r="C162" s="134" t="s">
         <v>21</v>
       </c>
-      <c r="D162" s="177">
+      <c r="D162" s="179">
         <f>F162*D158/100</f>
         <v>6000</v>
       </c>
-      <c r="E162" s="177"/>
+      <c r="E162" s="179"/>
       <c r="F162" s="153">
         <v>3</v>
       </c>
@@ -10864,6 +10911,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="K5:L5"/>
     <mergeCell ref="D161:E161"/>
     <mergeCell ref="D162:E162"/>
     <mergeCell ref="D156:E156"/>
@@ -10871,13 +10925,6 @@
     <mergeCell ref="D158:E158"/>
     <mergeCell ref="D159:E159"/>
     <mergeCell ref="D160:E160"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="I6:L6"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="K5:L5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -10906,29 +10953,29 @@
       <c r="A1" s="90">
         <v>152</v>
       </c>
-      <c r="B1" s="179" t="s">
+      <c r="B1" s="181" t="s">
         <v>106</v>
       </c>
-      <c r="C1" s="180"/>
-      <c r="D1" s="180"/>
-      <c r="E1" s="180"/>
-      <c r="F1" s="180"/>
-      <c r="G1" s="180"/>
-      <c r="H1" s="180"/>
+      <c r="C1" s="182"/>
+      <c r="D1" s="182"/>
+      <c r="E1" s="182"/>
+      <c r="F1" s="182"/>
+      <c r="G1" s="182"/>
+      <c r="H1" s="182"/>
     </row>
     <row r="2" spans="1:8" ht="15.75">
       <c r="A2" s="91" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="181" t="s">
+      <c r="B2" s="183" t="s">
         <v>108</v>
       </c>
-      <c r="C2" s="182"/>
-      <c r="D2" s="182"/>
-      <c r="E2" s="182"/>
-      <c r="F2" s="182"/>
-      <c r="G2" s="182"/>
-      <c r="H2" s="182"/>
+      <c r="C2" s="184"/>
+      <c r="D2" s="184"/>
+      <c r="E2" s="184"/>
+      <c r="F2" s="184"/>
+      <c r="G2" s="184"/>
+      <c r="H2" s="184"/>
     </row>
     <row r="3" spans="1:8" ht="31.5">
       <c r="A3" s="92"/>
@@ -10956,7 +11003,7 @@
     </row>
     <row r="4" spans="1:8" ht="16.5">
       <c r="A4" s="92"/>
-      <c r="B4" s="183" t="s">
+      <c r="B4" s="185" t="s">
         <v>116</v>
       </c>
       <c r="C4" s="94" t="s">
@@ -10979,7 +11026,7 @@
     </row>
     <row r="5" spans="1:8" ht="16.5">
       <c r="A5" s="92"/>
-      <c r="B5" s="184"/>
+      <c r="B5" s="186"/>
       <c r="C5" s="99" t="s">
         <v>119</v>
       </c>
@@ -11003,7 +11050,7 @@
     </row>
     <row r="6" spans="1:8" ht="16.5">
       <c r="A6" s="92"/>
-      <c r="B6" s="185" t="s">
+      <c r="B6" s="187" t="s">
         <v>120</v>
       </c>
       <c r="C6" s="96" t="s">
@@ -11027,7 +11074,7 @@
     </row>
     <row r="7" spans="1:8" ht="16.5">
       <c r="A7" s="92"/>
-      <c r="B7" s="186"/>
+      <c r="B7" s="188"/>
       <c r="C7" s="99" t="s">
         <v>123</v>
       </c>
@@ -11152,96 +11199,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="162" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="160"/>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160"/>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160"/>
-      <c r="I1" s="160"/>
-      <c r="J1" s="160"/>
-      <c r="K1" s="160"/>
-      <c r="L1" s="160"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
     </row>
     <row r="2" spans="1:12" ht="20.25">
-      <c r="A2" s="161" t="s">
+      <c r="A2" s="163" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="161"/>
-      <c r="C2" s="161"/>
-      <c r="D2" s="161"/>
-      <c r="E2" s="161"/>
-      <c r="F2" s="161"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="161"/>
-      <c r="I2" s="161"/>
-      <c r="J2" s="161"/>
-      <c r="K2" s="161"/>
-      <c r="L2" s="161"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
+      <c r="H2" s="163"/>
+      <c r="I2" s="163"/>
+      <c r="J2" s="163"/>
+      <c r="K2" s="163"/>
+      <c r="L2" s="163"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="160" t="s">
+      <c r="A3" s="162" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="160"/>
-      <c r="C3" s="160"/>
-      <c r="D3" s="160"/>
-      <c r="E3" s="160"/>
-      <c r="F3" s="160"/>
-      <c r="G3" s="160"/>
-      <c r="H3" s="160"/>
-      <c r="I3" s="160"/>
-      <c r="J3" s="160"/>
-      <c r="K3" s="160"/>
-      <c r="L3" s="160"/>
+      <c r="B3" s="162"/>
+      <c r="C3" s="162"/>
+      <c r="D3" s="162"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="162"/>
+      <c r="G3" s="162"/>
+      <c r="H3" s="162"/>
+      <c r="I3" s="162"/>
+      <c r="J3" s="162"/>
+      <c r="K3" s="162"/>
+      <c r="L3" s="162"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="162" t="s">
+      <c r="A4" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="162"/>
-      <c r="C4" s="162"/>
-      <c r="D4" s="162"/>
-      <c r="E4" s="162"/>
-      <c r="F4" s="162"/>
-      <c r="G4" s="162"/>
-      <c r="H4" s="162"/>
-      <c r="I4" s="162"/>
-      <c r="J4" s="162"/>
-      <c r="K4" s="162"/>
-      <c r="L4" s="162"/>
+      <c r="B4" s="164"/>
+      <c r="C4" s="164"/>
+      <c r="D4" s="164"/>
+      <c r="E4" s="164"/>
+      <c r="F4" s="164"/>
+      <c r="G4" s="164"/>
+      <c r="H4" s="164"/>
+      <c r="I4" s="164"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="164"/>
+      <c r="L4" s="164"/>
     </row>
     <row r="5" spans="1:12" ht="20.25">
       <c r="A5" s="6"/>
-      <c r="B5" s="187" t="s">
+      <c r="B5" s="158" t="s">
         <v>173</v>
       </c>
       <c r="H5" s="6"/>
-      <c r="K5" s="163" t="s">
+      <c r="K5" s="165" t="s">
         <v>101</v>
       </c>
-      <c r="L5" s="163"/>
+      <c r="L5" s="165"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="B6" s="164" t="s">
+      <c r="B6" s="166" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="164"/>
-      <c r="D6" s="164"/>
-      <c r="E6" s="164"/>
-      <c r="F6" s="164"/>
-      <c r="G6" s="164"/>
+      <c r="C6" s="166"/>
+      <c r="D6" s="166"/>
+      <c r="E6" s="166"/>
+      <c r="F6" s="166"/>
+      <c r="G6" s="166"/>
       <c r="H6" s="113"/>
-      <c r="I6" s="165" t="s">
+      <c r="I6" s="167" t="s">
         <v>174</v>
       </c>
-      <c r="J6" s="165"/>
-      <c r="K6" s="165"/>
-      <c r="L6" s="165"/>
+      <c r="J6" s="167"/>
+      <c r="K6" s="167"/>
+      <c r="L6" s="167"/>
     </row>
     <row r="7" spans="1:12">
       <c r="C7" s="5"/>
@@ -11364,6 +11411,7 @@
         <v>177</v>
       </c>
       <c r="D12" s="143">
+        <f>6</f>
         <v>6</v>
       </c>
       <c r="E12" s="130">
@@ -11386,7 +11434,7 @@
     </row>
     <row r="13" spans="1:12">
       <c r="B13" s="155"/>
-      <c r="C13" s="188" t="s">
+      <c r="C13" s="159" t="s">
         <v>178</v>
       </c>
       <c r="D13" s="1">
@@ -11585,11 +11633,11 @@
       <c r="C22" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="158">
+      <c r="D22" s="160">
         <f>+K20</f>
         <v>152392.78213992011</v>
       </c>
-      <c r="E22" s="158"/>
+      <c r="E22" s="160"/>
       <c r="G22" s="64"/>
       <c r="I22" s="2"/>
       <c r="J22" s="1"/>
@@ -11598,11 +11646,11 @@
       <c r="C23" s="134" t="s">
         <v>171</v>
       </c>
-      <c r="D23" s="158">
+      <c r="D23" s="160">
         <f>13%*D22</f>
         <v>19811.061678189613</v>
       </c>
-      <c r="E23" s="158"/>
+      <c r="E23" s="160"/>
       <c r="G23" s="64"/>
       <c r="I23" s="2"/>
       <c r="J23" s="1"/>
@@ -11611,11 +11659,11 @@
       <c r="C24" s="151" t="s">
         <v>172</v>
       </c>
-      <c r="D24" s="158">
+      <c r="D24" s="160">
         <f>SUM(D22:E23)</f>
         <v>172203.84381810972</v>
       </c>
-      <c r="E24" s="159"/>
+      <c r="E24" s="161"/>
       <c r="G24" s="62"/>
     </row>
   </sheetData>
@@ -11662,96 +11710,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="162" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="160"/>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160"/>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160"/>
-      <c r="I1" s="160"/>
-      <c r="J1" s="160"/>
-      <c r="K1" s="160"/>
-      <c r="L1" s="160"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
     </row>
     <row r="2" spans="1:12" ht="20.25">
-      <c r="A2" s="161" t="s">
+      <c r="A2" s="163" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="161"/>
-      <c r="C2" s="161"/>
-      <c r="D2" s="161"/>
-      <c r="E2" s="161"/>
-      <c r="F2" s="161"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="161"/>
-      <c r="I2" s="161"/>
-      <c r="J2" s="161"/>
-      <c r="K2" s="161"/>
-      <c r="L2" s="161"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
+      <c r="H2" s="163"/>
+      <c r="I2" s="163"/>
+      <c r="J2" s="163"/>
+      <c r="K2" s="163"/>
+      <c r="L2" s="163"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="160" t="s">
+      <c r="A3" s="162" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="160"/>
-      <c r="C3" s="160"/>
-      <c r="D3" s="160"/>
-      <c r="E3" s="160"/>
-      <c r="F3" s="160"/>
-      <c r="G3" s="160"/>
-      <c r="H3" s="160"/>
-      <c r="I3" s="160"/>
-      <c r="J3" s="160"/>
-      <c r="K3" s="160"/>
-      <c r="L3" s="160"/>
+      <c r="B3" s="162"/>
+      <c r="C3" s="162"/>
+      <c r="D3" s="162"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="162"/>
+      <c r="G3" s="162"/>
+      <c r="H3" s="162"/>
+      <c r="I3" s="162"/>
+      <c r="J3" s="162"/>
+      <c r="K3" s="162"/>
+      <c r="L3" s="162"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="162" t="s">
+      <c r="A4" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="162"/>
-      <c r="C4" s="162"/>
-      <c r="D4" s="162"/>
-      <c r="E4" s="162"/>
-      <c r="F4" s="162"/>
-      <c r="G4" s="162"/>
-      <c r="H4" s="162"/>
-      <c r="I4" s="162"/>
-      <c r="J4" s="162"/>
-      <c r="K4" s="162"/>
-      <c r="L4" s="162"/>
+      <c r="B4" s="164"/>
+      <c r="C4" s="164"/>
+      <c r="D4" s="164"/>
+      <c r="E4" s="164"/>
+      <c r="F4" s="164"/>
+      <c r="G4" s="164"/>
+      <c r="H4" s="164"/>
+      <c r="I4" s="164"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="164"/>
+      <c r="L4" s="164"/>
     </row>
     <row r="5" spans="1:12" ht="20.25">
       <c r="A5" s="6"/>
-      <c r="B5" s="187" t="s">
+      <c r="B5" s="158" t="s">
         <v>173</v>
       </c>
       <c r="H5" s="6"/>
-      <c r="K5" s="163" t="s">
+      <c r="K5" s="165" t="s">
         <v>101</v>
       </c>
-      <c r="L5" s="163"/>
+      <c r="L5" s="165"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="B6" s="164" t="s">
+      <c r="B6" s="166" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="164"/>
-      <c r="D6" s="164"/>
-      <c r="E6" s="164"/>
-      <c r="F6" s="164"/>
-      <c r="G6" s="164"/>
+      <c r="C6" s="166"/>
+      <c r="D6" s="166"/>
+      <c r="E6" s="166"/>
+      <c r="F6" s="166"/>
+      <c r="G6" s="166"/>
       <c r="H6" s="113"/>
-      <c r="I6" s="165" t="s">
+      <c r="I6" s="167" t="s">
         <v>174</v>
       </c>
-      <c r="J6" s="165"/>
-      <c r="K6" s="165"/>
-      <c r="L6" s="165"/>
+      <c r="J6" s="167"/>
+      <c r="K6" s="167"/>
+      <c r="L6" s="167"/>
     </row>
     <row r="7" spans="1:12">
       <c r="C7" s="5"/>
@@ -11896,7 +11944,7 @@
     </row>
     <row r="13" spans="1:12">
       <c r="B13" s="155"/>
-      <c r="C13" s="188" t="s">
+      <c r="C13" s="159" t="s">
         <v>178</v>
       </c>
       <c r="D13" s="1">
@@ -12130,7 +12178,7 @@
     </row>
     <row r="23" spans="2:12">
       <c r="B23" s="155"/>
-      <c r="C23" s="188" t="s">
+      <c r="C23" s="159" t="s">
         <v>178</v>
       </c>
       <c r="D23" s="1">
@@ -12329,11 +12377,11 @@
       <c r="C32" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D32" s="158">
+      <c r="D32" s="160">
         <f>+K30</f>
         <v>136152.90338529783</v>
       </c>
-      <c r="E32" s="158"/>
+      <c r="E32" s="160"/>
       <c r="G32" s="64"/>
       <c r="I32" s="2"/>
       <c r="J32" s="1"/>
@@ -12342,11 +12390,11 @@
       <c r="C33" s="134" t="s">
         <v>171</v>
       </c>
-      <c r="D33" s="158">
+      <c r="D33" s="160">
         <f>13%*D32</f>
         <v>17699.87744008872</v>
       </c>
-      <c r="E33" s="158"/>
+      <c r="E33" s="160"/>
       <c r="G33" s="64"/>
       <c r="I33" s="2"/>
       <c r="J33" s="1"/>
@@ -12355,11 +12403,11 @@
       <c r="C34" s="151" t="s">
         <v>172</v>
       </c>
-      <c r="D34" s="158">
+      <c r="D34" s="160">
         <f>SUM(D32:E33)</f>
         <v>153852.78082538655</v>
       </c>
-      <c r="E34" s="159"/>
+      <c r="E34" s="161"/>
       <c r="G34" s="62"/>
     </row>
   </sheetData>
@@ -12382,4 +12430,846 @@
     <oddHeader>&amp;RPage &amp;P of &amp;N</oddHeader>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D7B4C0F-01AE-4CFB-ACC2-61444527EF7A}">
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="3.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.85546875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="5.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.28515625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="162" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
+    </row>
+    <row r="2" spans="1:12" ht="20.25">
+      <c r="A2" s="163" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
+      <c r="H2" s="163"/>
+      <c r="I2" s="163"/>
+      <c r="J2" s="163"/>
+      <c r="K2" s="163"/>
+      <c r="L2" s="163"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="162" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="162"/>
+      <c r="C3" s="162"/>
+      <c r="D3" s="162"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="162"/>
+      <c r="G3" s="162"/>
+      <c r="H3" s="162"/>
+      <c r="I3" s="162"/>
+      <c r="J3" s="162"/>
+      <c r="K3" s="162"/>
+      <c r="L3" s="162"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="164" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="164"/>
+      <c r="C4" s="164"/>
+      <c r="D4" s="164"/>
+      <c r="E4" s="164"/>
+      <c r="F4" s="164"/>
+      <c r="G4" s="164"/>
+      <c r="H4" s="164"/>
+      <c r="I4" s="164"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="164"/>
+      <c r="L4" s="164"/>
+    </row>
+    <row r="5" spans="1:12" ht="20.25">
+      <c r="A5" s="6"/>
+      <c r="B5" s="158" t="s">
+        <v>180</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="K5" s="165" t="s">
+        <v>101</v>
+      </c>
+      <c r="L5" s="165"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="B6" s="166" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="166"/>
+      <c r="D6" s="166"/>
+      <c r="E6" s="166"/>
+      <c r="F6" s="166"/>
+      <c r="G6" s="166"/>
+      <c r="H6" s="113"/>
+      <c r="I6" s="167" t="s">
+        <v>182</v>
+      </c>
+      <c r="J6" s="167"/>
+      <c r="K6" s="167"/>
+      <c r="L6" s="167"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="C7" s="5"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
+      <c r="H7" s="113"/>
+      <c r="J7" s="114"/>
+      <c r="K7" s="113"/>
+      <c r="L7" s="8"/>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="2"/>
+      <c r="B8" s="120" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="121" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="156" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="154" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="154" t="s">
+        <v>4</v>
+      </c>
+      <c r="G8" s="154" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" s="154" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="156" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="154" t="s">
+        <v>8</v>
+      </c>
+      <c r="K8" s="154" t="s">
+        <v>9</v>
+      </c>
+      <c r="L8" s="157" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="57">
+      <c r="B9" s="155">
+        <v>1</v>
+      </c>
+      <c r="C9" s="128" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="129"/>
+      <c r="E9" s="130"/>
+      <c r="F9" s="130"/>
+      <c r="G9" s="135"/>
+      <c r="H9" s="130"/>
+      <c r="I9" s="129"/>
+      <c r="J9" s="130"/>
+      <c r="K9" s="130"/>
+      <c r="L9" s="131"/>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="B10" s="155"/>
+      <c r="C10" s="132" t="s">
+        <v>175</v>
+      </c>
+      <c r="D10" s="143">
+        <f>9</f>
+        <v>9</v>
+      </c>
+      <c r="E10" s="130">
+        <f>1.75/3.281</f>
+        <v>0.53337397135019804</v>
+      </c>
+      <c r="F10" s="130"/>
+      <c r="G10" s="135">
+        <f>3.5/3.281</f>
+        <v>1.0667479427003961</v>
+      </c>
+      <c r="H10" s="130">
+        <f>PRODUCT(D10:G10)</f>
+        <v>5.1207802796498738</v>
+      </c>
+      <c r="I10" s="129"/>
+      <c r="J10" s="130"/>
+      <c r="K10" s="130"/>
+      <c r="L10" s="131"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="B11" s="155"/>
+      <c r="C11" s="132" t="s">
+        <v>176</v>
+      </c>
+      <c r="D11" s="143">
+        <v>3</v>
+      </c>
+      <c r="E11" s="130">
+        <f>1.42/3.281</f>
+        <v>0.43279487960987501</v>
+      </c>
+      <c r="F11" s="130"/>
+      <c r="G11" s="135">
+        <v>1.2</v>
+      </c>
+      <c r="H11" s="130">
+        <f>PRODUCT(D11:G11)</f>
+        <v>1.55806156659555</v>
+      </c>
+      <c r="I11" s="129"/>
+      <c r="J11" s="130"/>
+      <c r="K11" s="130"/>
+      <c r="L11" s="131"/>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="B12" s="155"/>
+      <c r="C12" s="140"/>
+      <c r="D12" s="129"/>
+      <c r="E12" s="129"/>
+      <c r="F12" s="129"/>
+      <c r="G12" s="129"/>
+      <c r="H12" s="129">
+        <f>SUM(H10:H11)</f>
+        <v>6.6788418462454242</v>
+      </c>
+      <c r="I12" s="129" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" s="129">
+        <f>1.15*10663.63</f>
+        <v>12263.174499999997</v>
+      </c>
+      <c r="K12" s="129">
+        <f>H12*J12</f>
+        <v>81903.803018409788</v>
+      </c>
+      <c r="L12" s="131"/>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="B13" s="155"/>
+      <c r="C13" s="144"/>
+      <c r="D13" s="129"/>
+      <c r="E13" s="130"/>
+      <c r="F13" s="130"/>
+      <c r="G13" s="135"/>
+      <c r="H13" s="130"/>
+      <c r="I13" s="129"/>
+      <c r="J13" s="130"/>
+      <c r="K13" s="130"/>
+      <c r="L13" s="131"/>
+    </row>
+    <row r="14" spans="1:12" ht="33" customHeight="1">
+      <c r="B14" s="155">
+        <v>2</v>
+      </c>
+      <c r="C14" s="141" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="143">
+        <v>1</v>
+      </c>
+      <c r="E14" s="129"/>
+      <c r="F14" s="129"/>
+      <c r="G14" s="129"/>
+      <c r="H14" s="130">
+        <f>PRODUCT(D14:G14)</f>
+        <v>1</v>
+      </c>
+      <c r="I14" s="129" t="s">
+        <v>34</v>
+      </c>
+      <c r="J14" s="130">
+        <v>500</v>
+      </c>
+      <c r="K14" s="130">
+        <f>H14*J14</f>
+        <v>500</v>
+      </c>
+      <c r="L14" s="131"/>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="B15" s="148"/>
+      <c r="C15" s="149"/>
+      <c r="D15" s="129"/>
+      <c r="E15" s="130"/>
+      <c r="F15" s="130"/>
+      <c r="G15" s="130"/>
+      <c r="H15" s="130"/>
+      <c r="I15" s="129"/>
+      <c r="J15" s="130"/>
+      <c r="K15" s="150">
+        <f>SUM(K9:K14)</f>
+        <v>82403.803018409788</v>
+      </c>
+      <c r="L15" s="151"/>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="C16" s="9"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="118"/>
+      <c r="L16" s="8"/>
+    </row>
+    <row r="17" spans="3:10">
+      <c r="C17" s="134" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="160">
+        <f>+K15</f>
+        <v>82403.803018409788</v>
+      </c>
+      <c r="E17" s="160"/>
+      <c r="G17" s="64"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="3:10">
+      <c r="C18" s="134" t="s">
+        <v>171</v>
+      </c>
+      <c r="D18" s="160">
+        <f>13%*D17</f>
+        <v>10712.494392393273</v>
+      </c>
+      <c r="E18" s="160"/>
+      <c r="G18" s="64"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="3:10">
+      <c r="C19" s="151" t="s">
+        <v>172</v>
+      </c>
+      <c r="D19" s="160">
+        <f>SUM(D17:E18)</f>
+        <v>93116.297410803061</v>
+      </c>
+      <c r="E19" s="161"/>
+      <c r="G19" s="62"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="I6:L6"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.511811023622047" right="0.511811023622047" top="0.39370078740157499" bottom="0.70866141732283505" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" scale="80" fitToHeight="2" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;RPage &amp;P of &amp;N</oddHeader>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EDFBFC3-6CBB-4427-8EDC-BA8E637E0A67}">
+  <dimension ref="A1:L22"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="3.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.85546875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="5.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.28515625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="162" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
+    </row>
+    <row r="2" spans="1:12" ht="20.25">
+      <c r="A2" s="163" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
+      <c r="H2" s="163"/>
+      <c r="I2" s="163"/>
+      <c r="J2" s="163"/>
+      <c r="K2" s="163"/>
+      <c r="L2" s="163"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="162" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="162"/>
+      <c r="C3" s="162"/>
+      <c r="D3" s="162"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="162"/>
+      <c r="G3" s="162"/>
+      <c r="H3" s="162"/>
+      <c r="I3" s="162"/>
+      <c r="J3" s="162"/>
+      <c r="K3" s="162"/>
+      <c r="L3" s="162"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="164" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="164"/>
+      <c r="C4" s="164"/>
+      <c r="D4" s="164"/>
+      <c r="E4" s="164"/>
+      <c r="F4" s="164"/>
+      <c r="G4" s="164"/>
+      <c r="H4" s="164"/>
+      <c r="I4" s="164"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="164"/>
+      <c r="L4" s="164"/>
+    </row>
+    <row r="5" spans="1:12" ht="20.25">
+      <c r="A5" s="6"/>
+      <c r="B5" s="158" t="s">
+        <v>181</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="K5" s="165" t="s">
+        <v>101</v>
+      </c>
+      <c r="L5" s="165"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="B6" s="166" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="166"/>
+      <c r="D6" s="166"/>
+      <c r="E6" s="166"/>
+      <c r="F6" s="166"/>
+      <c r="G6" s="166"/>
+      <c r="H6" s="113"/>
+      <c r="I6" s="167" t="s">
+        <v>182</v>
+      </c>
+      <c r="J6" s="167"/>
+      <c r="K6" s="167"/>
+      <c r="L6" s="167"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="C7" s="5"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
+      <c r="H7" s="113"/>
+      <c r="J7" s="114"/>
+      <c r="K7" s="113"/>
+      <c r="L7" s="8"/>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="2"/>
+      <c r="B8" s="120" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="121" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="156" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="154" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="154" t="s">
+        <v>4</v>
+      </c>
+      <c r="G8" s="154" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" s="154" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="156" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="154" t="s">
+        <v>8</v>
+      </c>
+      <c r="K8" s="154" t="s">
+        <v>9</v>
+      </c>
+      <c r="L8" s="157" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="57">
+      <c r="B9" s="155">
+        <v>1</v>
+      </c>
+      <c r="C9" s="128" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="129"/>
+      <c r="E9" s="130"/>
+      <c r="F9" s="130"/>
+      <c r="G9" s="135"/>
+      <c r="H9" s="130"/>
+      <c r="I9" s="129"/>
+      <c r="J9" s="130"/>
+      <c r="K9" s="130"/>
+      <c r="L9" s="131"/>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="B10" s="155"/>
+      <c r="C10" s="132" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="143">
+        <f>6+2</f>
+        <v>8</v>
+      </c>
+      <c r="E10" s="130">
+        <f>1.75/3.281</f>
+        <v>0.53337397135019804</v>
+      </c>
+      <c r="F10" s="130"/>
+      <c r="G10" s="135">
+        <f>3.5/3.281</f>
+        <v>1.0667479427003961</v>
+      </c>
+      <c r="H10" s="130">
+        <f>PRODUCT(D10:G10)</f>
+        <v>4.5518046930221097</v>
+      </c>
+      <c r="I10" s="129"/>
+      <c r="J10" s="130"/>
+      <c r="K10" s="130"/>
+      <c r="L10" s="131"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="B11" s="155"/>
+      <c r="C11" s="159" t="s">
+        <v>178</v>
+      </c>
+      <c r="D11" s="143">
+        <f>1+1+1</f>
+        <v>3</v>
+      </c>
+      <c r="E11" s="130">
+        <f>1.667/3.281</f>
+        <v>0.50807680585187442</v>
+      </c>
+      <c r="F11" s="130"/>
+      <c r="G11" s="135">
+        <f>2.083/3.281</f>
+        <v>0.63486741846997874</v>
+      </c>
+      <c r="H11" s="130">
+        <f t="shared" ref="H11:H14" si="0">PRODUCT(D11:G11)</f>
+        <v>0.96768423034695628</v>
+      </c>
+      <c r="I11" s="129"/>
+      <c r="J11" s="130"/>
+      <c r="K11" s="130"/>
+      <c r="L11" s="131"/>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="B12" s="155"/>
+      <c r="C12" s="132"/>
+      <c r="D12" s="143">
+        <f>1+1</f>
+        <v>2</v>
+      </c>
+      <c r="E12" s="130">
+        <f>1.75/3.281</f>
+        <v>0.53337397135019804</v>
+      </c>
+      <c r="F12" s="130"/>
+      <c r="G12" s="135">
+        <f>2.083/3.281</f>
+        <v>0.63486741846997874</v>
+      </c>
+      <c r="H12" s="130">
+        <f t="shared" si="0"/>
+        <v>0.6772435125403613</v>
+      </c>
+      <c r="I12" s="129"/>
+      <c r="J12" s="130"/>
+      <c r="K12" s="130"/>
+      <c r="L12" s="131"/>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="B13" s="155"/>
+      <c r="C13" s="132" t="s">
+        <v>179</v>
+      </c>
+      <c r="D13" s="143">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="E13" s="130">
+        <f>1.75/3.281</f>
+        <v>0.53337397135019804</v>
+      </c>
+      <c r="F13" s="130"/>
+      <c r="G13" s="135">
+        <f>1.42/3.281</f>
+        <v>0.43279487960987501</v>
+      </c>
+      <c r="H13" s="130">
+        <f t="shared" si="0"/>
+        <v>0.23084152371754987</v>
+      </c>
+      <c r="I13" s="129"/>
+      <c r="J13" s="130"/>
+      <c r="K13" s="130"/>
+      <c r="L13" s="131"/>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="B14" s="155"/>
+      <c r="C14" s="132"/>
+      <c r="D14" s="143">
+        <v>2</v>
+      </c>
+      <c r="E14" s="130">
+        <f>1.42/3.281</f>
+        <v>0.43279487960987501</v>
+      </c>
+      <c r="F14" s="130"/>
+      <c r="G14" s="135">
+        <f>1.583/3.281</f>
+        <v>0.4824748552270649</v>
+      </c>
+      <c r="H14" s="130">
+        <f t="shared" si="0"/>
+        <v>0.41762529376557883</v>
+      </c>
+      <c r="I14" s="129"/>
+      <c r="J14" s="130"/>
+      <c r="K14" s="130"/>
+      <c r="L14" s="131"/>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="B15" s="155"/>
+      <c r="C15" s="140"/>
+      <c r="D15" s="129"/>
+      <c r="E15" s="129"/>
+      <c r="F15" s="129"/>
+      <c r="G15" s="129"/>
+      <c r="H15" s="129">
+        <f>SUM(H10:H14)</f>
+        <v>6.8451992533925559</v>
+      </c>
+      <c r="I15" s="129" t="s">
+        <v>90</v>
+      </c>
+      <c r="J15" s="129">
+        <f>1.15*10663.63</f>
+        <v>12263.174499999997</v>
+      </c>
+      <c r="K15" s="129">
+        <f>H15*J15</f>
+        <v>83943.872931622609</v>
+      </c>
+      <c r="L15" s="131"/>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="B16" s="155"/>
+      <c r="C16" s="144"/>
+      <c r="D16" s="129"/>
+      <c r="E16" s="130"/>
+      <c r="F16" s="130"/>
+      <c r="G16" s="135"/>
+      <c r="H16" s="130"/>
+      <c r="I16" s="129"/>
+      <c r="J16" s="130"/>
+      <c r="K16" s="130"/>
+      <c r="L16" s="131"/>
+    </row>
+    <row r="17" spans="2:12" ht="33" customHeight="1">
+      <c r="B17" s="155">
+        <v>2</v>
+      </c>
+      <c r="C17" s="141" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" s="143">
+        <v>1</v>
+      </c>
+      <c r="E17" s="129"/>
+      <c r="F17" s="129"/>
+      <c r="G17" s="129"/>
+      <c r="H17" s="130">
+        <f>PRODUCT(D17:G17)</f>
+        <v>1</v>
+      </c>
+      <c r="I17" s="129" t="s">
+        <v>34</v>
+      </c>
+      <c r="J17" s="130">
+        <v>500</v>
+      </c>
+      <c r="K17" s="130">
+        <f>H17*J17</f>
+        <v>500</v>
+      </c>
+      <c r="L17" s="131"/>
+    </row>
+    <row r="18" spans="2:12">
+      <c r="B18" s="148"/>
+      <c r="C18" s="149"/>
+      <c r="D18" s="129"/>
+      <c r="E18" s="130"/>
+      <c r="F18" s="130"/>
+      <c r="G18" s="130"/>
+      <c r="H18" s="130"/>
+      <c r="I18" s="129"/>
+      <c r="J18" s="130"/>
+      <c r="K18" s="150">
+        <f>SUM(K9:K17)</f>
+        <v>84443.872931622609</v>
+      </c>
+      <c r="L18" s="151"/>
+    </row>
+    <row r="19" spans="2:12">
+      <c r="C19" s="9"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="118"/>
+      <c r="L19" s="8"/>
+    </row>
+    <row r="20" spans="2:12">
+      <c r="C20" s="134" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="160">
+        <f>+K18</f>
+        <v>84443.872931622609</v>
+      </c>
+      <c r="E20" s="160"/>
+      <c r="G20" s="64"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="2:12">
+      <c r="C21" s="134" t="s">
+        <v>171</v>
+      </c>
+      <c r="D21" s="160">
+        <f>13%*D20</f>
+        <v>10977.703481110939</v>
+      </c>
+      <c r="E21" s="160"/>
+      <c r="G21" s="64"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="1"/>
+    </row>
+    <row r="22" spans="2:12">
+      <c r="C22" s="151" t="s">
+        <v>172</v>
+      </c>
+      <c r="D22" s="160">
+        <f>SUM(D20:E21)</f>
+        <v>95421.576412733542</v>
+      </c>
+      <c r="E22" s="161"/>
+      <c r="G22" s="62"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="I6:L6"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.511811023622047" right="0.511811023622047" top="0.39370078740157499" bottom="0.70866141732283505" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" scale="80" fitToHeight="2" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;RPage &amp;P of &amp;N</oddHeader>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>